<commit_message>
feat: load client register from Stranke.xlsx
</commit_message>
<xml_diff>
--- a/public/assets/Stranke.xlsx
+++ b/public/assets/Stranke.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\talpas-invoice\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{571E9BBF-0DA6-43D3-89BF-7B08D7F22269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36503D06-68EB-4113-B67F-8E9E300BDE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{54F47D17-901F-4DA7-82BF-452E61896D1B}"/>
+    <workbookView xWindow="0" yWindow="45" windowWidth="25365" windowHeight="15345" xr2:uid="{54F47D17-901F-4DA7-82BF-452E61896D1B}"/>
   </bookViews>
   <sheets>
     <sheet name="query" sheetId="1" r:id="rId1"/>
@@ -3237,6 +3237,7 @@
     <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8901,20 +8902,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44b6e255-9bec-4b65-ada2-b42ea9c0f358" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44b6e255-9bec-4b65-ada2-b42ea9c0f358" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8936,6 +8937,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3560CBC-637F-42C1-B146-9EED4519BB73}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -8949,12 +8958,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix: UL/UP izključi VIS, UL postavke brez zneska, priloge po abecedi
- filterForUniType: VIS stranke nikoli pod UL/UP; UL kratice iz UL_specifika
  so avtoritativne (varuje FA, NTF ipd. pred napačno VIS-klasifikacijo)
- UL_specifika: podpora vrsticam brez mesečnega zneska (UL VO/STAT/BM) –
  izpiše se samo postavka s praznimi zneski; kratica iz cele vrednosti
- normKratica/normUl tolerirata pomišljaje ("UL VO" = "UL-VO")
- priloge (specifikacije) razvrščene: Rektorat prvi, ostale po abecedi

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/assets/Stranke.xlsx
+++ b/public/assets/Stranke.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\talpas-invoice\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDDAC60-D913-4757-A317-BE5E4BDCB17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBE66C2-D3E2-48F6-B02A-DA88A052FA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{54F47D17-901F-4DA7-82BF-452E61896D1B}"/>
   </bookViews>
@@ -3259,6 +3259,7 @@
     <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
fix: date format, sklic, clients without entries
- Standardni Word izvoz: datumi v obliki d.M.yyyy (formatObdobje) za
  datumRacuna, rokPlacila, obdobjeOd, obdobjeDo
- Sklic: odstranjen podvojeni "SI 00" (predloga ze vsebuje prefiks)
- Stranke z mesecnim pavsalom (>0, stolpec F prazen) brez vnosov v Excelu
  se prikazejo v seznamu; izvoz vsebuje samo vrstico vzdrzevanja (brez priloge)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/assets/Stranke.xlsx
+++ b/public/assets/Stranke.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\talpas-invoice\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBE66C2-D3E2-48F6-B02A-DA88A052FA50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AD371E-A6F5-43B4-9D28-75FC80C7B1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{54F47D17-901F-4DA7-82BF-452E61896D1B}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1290" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="749">
   <si>
     <t>Kratica</t>
   </si>
@@ -2275,6 +2275,9 @@
   </si>
   <si>
     <t>VIS</t>
+  </si>
+  <si>
+    <t>318</t>
   </si>
 </sst>
 </file>
@@ -3363,9 +3366,15 @@
         <v>15</v>
       </c>
       <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>718</v>
+      </c>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -5961,9 +5970,15 @@
         <v>358</v>
       </c>
       <c r="F122" s="1"/>
-      <c r="G122" s="1"/>
-      <c r="H122" s="1"/>
-      <c r="I122" s="1"/>
+      <c r="G122" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>718</v>
+      </c>
       <c r="J122" s="1"/>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.25">
@@ -6723,9 +6738,15 @@
       </c>
       <c r="E158" s="1"/>
       <c r="F158" s="1"/>
-      <c r="G158" s="1"/>
-      <c r="H158" s="1"/>
-      <c r="I158" s="1"/>
+      <c r="G158" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="H158" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="I158" s="1" t="s">
+        <v>718</v>
+      </c>
       <c r="J158" s="1"/>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.25">
@@ -9123,20 +9144,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44b6e255-9bec-4b65-ada2-b42ea9c0f358" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44b6e255-9bec-4b65-ada2-b42ea9c0f358" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9158,14 +9179,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3560CBC-637F-42C1-B146-9EED4519BB73}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -9179,4 +9192,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix: partial name matching
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/assets/Stranke.xlsx
+++ b/public/assets/Stranke.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\talpas-invoice\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CD5081-E1E5-47F5-AA57-438E6A329A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF58EF7-DB09-49C9-BF64-BE947CEF21B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{54F47D17-901F-4DA7-82BF-452E61896D1B}"/>
   </bookViews>
@@ -2252,13 +2252,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A37B9E62-4060-4509-B0D0-60F912CE029E}" name="Table_query" displayName="Table_query" ref="A1:O127" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:O127" xr:uid="{A37B9E62-4060-4509-B0D0-60F912CE029E}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="VIS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:O127" xr:uid="{A37B9E62-4060-4509-B0D0-60F912CE029E}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{B3D59791-FB16-42CB-A5D4-2A3DA647622B}" uniqueName="Title" name="Kratica" queryTableFieldId="1" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{B7A63C42-317B-4372-8AF6-7B74693BE5F3}" uniqueName="Naziva" name="Naziv" queryTableFieldId="6" dataDxfId="13"/>
@@ -2658,7 +2652,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -2728,7 +2722,7 @@
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -2763,7 +2757,7 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -2798,7 +2792,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -2826,7 +2820,7 @@
       <c r="O6" s="1"/>
       <c r="Q6" s="6"/>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -2864,7 +2858,7 @@
       <c r="O7" s="1"/>
       <c r="Q7" s="6"/>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -2902,7 +2896,7 @@
       <c r="O8" s="1"/>
       <c r="Q8" s="6"/>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -2978,7 +2972,7 @@
       <c r="N10" s="10"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
@@ -3011,7 +3005,7 @@
       <c r="N11" s="10"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>36</v>
       </c>
@@ -3044,7 +3038,7 @@
       <c r="N12" s="10"/>
       <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>38</v>
       </c>
@@ -3114,7 +3108,7 @@
       <c r="N14" s="10"/>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>43</v>
       </c>
@@ -3141,7 +3135,7 @@
       <c r="N15" s="10"/>
       <c r="O15" s="1"/>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>46</v>
       </c>
@@ -3178,7 +3172,7 @@
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>492</v>
       </c>
@@ -3211,7 +3205,7 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>51</v>
       </c>
@@ -3312,7 +3306,7 @@
       <c r="N20" s="10"/>
       <c r="O20" s="1"/>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>55</v>
       </c>
@@ -3345,7 +3339,7 @@
       <c r="N21" s="10"/>
       <c r="O21" s="1"/>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>58</v>
       </c>
@@ -3415,7 +3409,7 @@
       <c r="N23" s="10"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>63</v>
       </c>
@@ -3514,7 +3508,7 @@
       <c r="O26" s="7"/>
       <c r="P26" s="9"/>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>69</v>
       </c>
@@ -3552,7 +3546,7 @@
       <c r="O27" s="1"/>
       <c r="P27" s="6"/>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>72</v>
       </c>
@@ -3612,7 +3606,7 @@
       <c r="N29" s="1"/>
       <c r="O29" s="1"/>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>76</v>
       </c>
@@ -3789,7 +3783,7 @@
       <c r="O34" s="10"/>
       <c r="Q34" s="6"/>
     </row>
-    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>86</v>
       </c>
@@ -3825,7 +3819,7 @@
       <c r="O35" s="1"/>
       <c r="Q35" s="6"/>
     </row>
-    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>88</v>
       </c>
@@ -3900,7 +3894,7 @@
       <c r="N37" s="1"/>
       <c r="O37" s="10"/>
     </row>
-    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>94</v>
       </c>
@@ -3999,7 +3993,7 @@
       <c r="N40" s="1"/>
       <c r="O40" s="10"/>
     </row>
-    <row r="41" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>102</v>
       </c>
@@ -4036,7 +4030,7 @@
       <c r="N41" s="1"/>
       <c r="O41" s="10"/>
     </row>
-    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>105</v>
       </c>
@@ -4073,7 +4067,7 @@
       <c r="N42" s="1"/>
       <c r="O42" s="10"/>
     </row>
-    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>108</v>
       </c>
@@ -4110,7 +4104,7 @@
       <c r="N43" s="1"/>
       <c r="O43" s="1"/>
     </row>
-    <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>111</v>
       </c>
@@ -4186,7 +4180,7 @@
       <c r="N45" s="1"/>
       <c r="O45" s="10"/>
     </row>
-    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>116</v>
       </c>
@@ -4335,7 +4329,7 @@
       <c r="O49" s="1"/>
       <c r="P49" s="6"/>
     </row>
-    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>126</v>
       </c>
@@ -4370,7 +4364,7 @@
       <c r="O50" s="1"/>
       <c r="P50" s="6"/>
     </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>128</v>
       </c>
@@ -4407,7 +4401,7 @@
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
     </row>
-    <row r="52" spans="1:17" s="16" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>131</v>
       </c>
@@ -4544,7 +4538,7 @@
       <c r="O55" s="1"/>
       <c r="Q55" s="6"/>
     </row>
-    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>141</v>
       </c>
@@ -4572,7 +4566,7 @@
       <c r="O56" s="1"/>
       <c r="Q56" s="6"/>
     </row>
-    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>144</v>
       </c>
@@ -4608,7 +4602,7 @@
       <c r="O57" s="1"/>
       <c r="Q57" s="6"/>
     </row>
-    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>147</v>
       </c>
@@ -4636,7 +4630,7 @@
       <c r="O58" s="1"/>
       <c r="Q58" s="6"/>
     </row>
-    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>148</v>
       </c>
@@ -4670,7 +4664,7 @@
       <c r="O59" s="1"/>
       <c r="Q59" s="6"/>
     </row>
-    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>150</v>
       </c>
@@ -4704,7 +4698,7 @@
       <c r="O60" s="1"/>
       <c r="Q60" s="6"/>
     </row>
-    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>153</v>
       </c>
@@ -4732,7 +4726,7 @@
       <c r="O61" s="1"/>
       <c r="Q61" s="6"/>
     </row>
-    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>155</v>
       </c>
@@ -4760,7 +4754,7 @@
       <c r="O62" s="1"/>
       <c r="Q62" s="6"/>
     </row>
-    <row r="63" spans="1:17" s="16" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
         <v>159</v>
       </c>
@@ -4785,7 +4779,7 @@
       <c r="N63" s="14"/>
       <c r="O63" s="14"/>
     </row>
-    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>161</v>
       </c>
@@ -4813,7 +4807,7 @@
       <c r="O64" s="1"/>
       <c r="Q64" s="6"/>
     </row>
-    <row r="65" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>164</v>
       </c>
@@ -4841,7 +4835,7 @@
       <c r="O65" s="1"/>
       <c r="Q65" s="6"/>
     </row>
-    <row r="66" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>168</v>
       </c>
@@ -4875,7 +4869,7 @@
       <c r="O66" s="1"/>
       <c r="Q66" s="6"/>
     </row>
-    <row r="67" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>171</v>
       </c>
@@ -4941,7 +4935,7 @@
       <c r="O68" s="1"/>
       <c r="Q68" s="6"/>
     </row>
-    <row r="69" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>173</v>
       </c>
@@ -4975,7 +4969,7 @@
       <c r="O69" s="1"/>
       <c r="R69" s="12"/>
     </row>
-    <row r="70" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>175</v>
       </c>
@@ -5009,7 +5003,7 @@
       <c r="O70" s="1"/>
       <c r="Q70" s="6"/>
     </row>
-    <row r="71" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>177</v>
       </c>
@@ -5085,7 +5079,7 @@
       <c r="O72" s="1"/>
       <c r="Q72" s="6"/>
     </row>
-    <row r="73" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>182</v>
       </c>
@@ -5119,7 +5113,7 @@
       <c r="O73" s="1"/>
       <c r="Q73" s="6"/>
     </row>
-    <row r="74" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>185</v>
       </c>
@@ -5156,7 +5150,7 @@
       <c r="N74" s="1"/>
       <c r="O74" s="1"/>
     </row>
-    <row r="75" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>188</v>
       </c>
@@ -5190,7 +5184,7 @@
       <c r="O75" s="1"/>
       <c r="Q75" s="6"/>
     </row>
-    <row r="76" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>190</v>
       </c>
@@ -5289,7 +5283,7 @@
       <c r="N78" s="1"/>
       <c r="O78" s="1"/>
     </row>
-    <row r="79" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>195</v>
       </c>
@@ -5316,7 +5310,7 @@
       <c r="N79" s="1"/>
       <c r="O79" s="1"/>
     </row>
-    <row r="80" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>197</v>
       </c>
@@ -5344,7 +5338,7 @@
       <c r="O80" s="1"/>
       <c r="Q80" s="6"/>
     </row>
-    <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>199</v>
       </c>
@@ -5378,7 +5372,7 @@
       <c r="O81" s="1"/>
       <c r="R81" s="6"/>
     </row>
-    <row r="82" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>200</v>
       </c>
@@ -5416,7 +5410,7 @@
       </c>
       <c r="R82" s="6"/>
     </row>
-    <row r="83" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>201</v>
       </c>
@@ -5452,7 +5446,7 @@
       <c r="O83" s="1"/>
       <c r="Q83" s="6"/>
     </row>
-    <row r="84" spans="1:18" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
         <v>204</v>
       </c>
@@ -5478,7 +5472,7 @@
       <c r="O84" s="7"/>
       <c r="Q84" s="9"/>
     </row>
-    <row r="85" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>207</v>
       </c>
@@ -5513,7 +5507,7 @@
       <c r="N85" s="1"/>
       <c r="O85" s="1"/>
     </row>
-    <row r="86" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>208</v>
       </c>
@@ -5588,7 +5582,7 @@
       <c r="O87" s="1"/>
       <c r="P87" s="6"/>
     </row>
-    <row r="88" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>212</v>
       </c>
@@ -5617,7 +5611,7 @@
       <c r="P88" s="6"/>
       <c r="Q88" s="6"/>
     </row>
-    <row r="89" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>214</v>
       </c>
@@ -5654,7 +5648,7 @@
       <c r="N89" s="1"/>
       <c r="O89" s="1"/>
     </row>
-    <row r="90" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>217</v>
       </c>
@@ -5682,7 +5676,7 @@
       <c r="O90" s="1"/>
       <c r="R90" s="12"/>
     </row>
-    <row r="91" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>440</v>
       </c>
@@ -5710,7 +5704,7 @@
       <c r="O91" s="1"/>
       <c r="Q91" s="6"/>
     </row>
-    <row r="92" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>218</v>
       </c>
@@ -5744,7 +5738,7 @@
       <c r="O92" s="1"/>
       <c r="Q92" s="6"/>
     </row>
-    <row r="93" spans="1:18" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>220</v>
       </c>
@@ -5775,7 +5769,7 @@
       <c r="N93" s="7"/>
       <c r="O93" s="7"/>
     </row>
-    <row r="94" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>224</v>
       </c>
@@ -5802,7 +5796,7 @@
       <c r="N94" s="1"/>
       <c r="O94" s="1"/>
     </row>
-    <row r="95" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>227</v>
       </c>
@@ -5836,7 +5830,7 @@
       <c r="O95" s="1"/>
       <c r="Q95" s="6"/>
     </row>
-    <row r="96" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>228</v>
       </c>
@@ -5870,7 +5864,7 @@
       <c r="O96" s="1"/>
       <c r="Q96" s="6"/>
     </row>
-    <row r="97" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>231</v>
       </c>
@@ -5898,7 +5892,7 @@
       <c r="O97" s="1"/>
       <c r="Q97" s="6"/>
     </row>
-    <row r="98" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>234</v>
       </c>
@@ -5935,7 +5929,7 @@
       <c r="N98" s="1"/>
       <c r="O98" s="1"/>
     </row>
-    <row r="99" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>237</v>
       </c>
@@ -5969,7 +5963,7 @@
       <c r="O99" s="1"/>
       <c r="Q99" s="6"/>
     </row>
-    <row r="100" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>241</v>
       </c>
@@ -6005,7 +5999,7 @@
       <c r="O100" s="1"/>
       <c r="Q100" s="6"/>
     </row>
-    <row r="101" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>243</v>
       </c>
@@ -6040,7 +6034,7 @@
       <c r="N101" s="1"/>
       <c r="O101" s="1"/>
     </row>
-    <row r="102" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>246</v>
       </c>
@@ -6074,7 +6068,7 @@
       <c r="O102" s="1"/>
       <c r="Q102" s="12"/>
     </row>
-    <row r="103" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>247</v>
       </c>
@@ -6112,7 +6106,7 @@
       <c r="O103" s="1"/>
       <c r="Q103" s="6"/>
     </row>
-    <row r="104" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>249</v>
       </c>
@@ -6147,7 +6141,7 @@
       <c r="N104" s="1"/>
       <c r="O104" s="1"/>
     </row>
-    <row r="105" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>251</v>
       </c>
@@ -6182,7 +6176,7 @@
       <c r="N105" s="1"/>
       <c r="O105" s="1"/>
     </row>
-    <row r="106" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>253</v>
       </c>
@@ -6217,7 +6211,7 @@
       <c r="N106" s="1"/>
       <c r="O106" s="1"/>
     </row>
-    <row r="107" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>255</v>
       </c>
@@ -6253,7 +6247,7 @@
       <c r="O107" s="1"/>
       <c r="Q107" s="6"/>
     </row>
-    <row r="108" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>257</v>
       </c>
@@ -6466,7 +6460,7 @@
       <c r="N113" s="1"/>
       <c r="O113" s="1"/>
     </row>
-    <row r="114" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>261</v>
       </c>
@@ -6493,7 +6487,7 @@
       <c r="N114" s="1"/>
       <c r="O114" s="1"/>
     </row>
-    <row r="115" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>263</v>
       </c>
@@ -6530,7 +6524,7 @@
       <c r="N115" s="1"/>
       <c r="O115" s="1"/>
     </row>
-    <row r="116" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>266</v>
       </c>
@@ -6755,7 +6749,7 @@
       <c r="O121" s="1"/>
       <c r="Q121" s="6"/>
     </row>
-    <row r="122" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>278</v>
       </c>
@@ -6791,7 +6785,7 @@
       <c r="O122" s="1"/>
       <c r="Q122" s="6"/>
     </row>
-    <row r="123" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>279</v>
       </c>
@@ -6825,7 +6819,7 @@
       <c r="O123" s="1"/>
       <c r="Q123" s="6"/>
     </row>
-    <row r="124" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>282</v>
       </c>
@@ -6897,7 +6891,7 @@
       <c r="O125" s="1"/>
       <c r="Q125" s="6"/>
     </row>
-    <row r="126" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>285</v>
       </c>
@@ -6934,7 +6928,7 @@
       <c r="N126" s="1"/>
       <c r="O126" s="1"/>
     </row>
-    <row r="127" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>288</v>
       </c>
@@ -6983,6 +6977,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B8424CE85351F64589369729664893D7" ma:contentTypeVersion="5" ma:contentTypeDescription="Ustvari nov dokument." ma:contentTypeScope="" ma:versionID="1ac781d2aabc82e157e45a1e96b6231b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44b6e255-9bec-4b65-ada2-b42ea9c0f358" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79a5782f82df6e133ce65d5df1a4d33b" ns3:_="">
     <xsd:import namespace="44b6e255-9bec-4b65-ada2-b42ea9c0f358"/>
@@ -7132,15 +7135,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3560CBC-637F-42C1-B146-9EED4519BB73}">
   <ds:schemaRefs>
@@ -7158,6 +7152,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EFA213E-BAB9-41D9-8FDD-B1DDC4C0B256}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7173,12 +7175,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: slovenian spellcheck in word export
</commit_message>
<xml_diff>
--- a/public/assets/Stranke.xlsx
+++ b/public/assets/Stranke.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\talpas-invoice\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF58EF7-DB09-49C9-BF64-BE947CEF21B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F9E391-5435-4053-A80E-BA349BE4C586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{54F47D17-901F-4DA7-82BF-452E61896D1B}"/>
   </bookViews>
@@ -6969,23 +6969,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44b6e255-9bec-4b65-ada2-b42ea9c0f358" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B8424CE85351F64589369729664893D7" ma:contentTypeVersion="5" ma:contentTypeDescription="Ustvari nov dokument." ma:contentTypeScope="" ma:versionID="1ac781d2aabc82e157e45a1e96b6231b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44b6e255-9bec-4b65-ada2-b42ea9c0f358" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79a5782f82df6e133ce65d5df1a4d33b" ns3:_="">
     <xsd:import namespace="44b6e255-9bec-4b65-ada2-b42ea9c0f358"/>
@@ -7135,7 +7118,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44b6e255-9bec-4b65-ada2-b42ea9c0f358" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EFA213E-BAB9-41D9-8FDD-B1DDC4C0B256}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="44b6e255-9bec-4b65-ada2-b42ea9c0f358"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3560CBC-637F-42C1-B146-9EED4519BB73}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -7151,28 +7169,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF107626-ADC0-42BC-82E5-E38C6154BC12}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EFA213E-BAB9-41D9-8FDD-B1DDC4C0B256}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="44b6e255-9bec-4b65-ada2-b42ea9c0f358"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>